<commit_message>
Add new fields: property name, tech name, AI summary, caller info, full detail view
</commit_message>
<xml_diff>
--- a/Properties.xlsx
+++ b/Properties.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\PycharmProjects\WOApp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\PycharmProjects\WorkOrderBot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F32A6C9A-37B5-40C4-97EE-FFC963451007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118E810F-A0C4-4A83-B940-FE51390FFC7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8BB1177E-FB22-4B22-B7F4-415662DFB70E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="46">
   <si>
     <t>Property</t>
   </si>
@@ -165,6 +165,18 @@
   </si>
   <si>
     <t>Murals on Niazuma</t>
+  </si>
+  <si>
+    <t>Yardi</t>
+  </si>
+  <si>
+    <t>asmith</t>
+  </si>
+  <si>
+    <t>dhall</t>
+  </si>
+  <si>
+    <t>morton</t>
   </si>
 </sst>
 </file>
@@ -569,15 +581,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42840889-76A4-4A3F-9F79-7860A1155E34}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.7109375" style="4" customWidth="1"/>
-    <col min="2" max="4" width="20.5703125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="20.5703125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -585,16 +597,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>79800</v>
       </c>
@@ -602,16 +617,19 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>79200</v>
       </c>
@@ -619,16 +637,19 @@
         <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>75000</v>
       </c>
@@ -636,16 +657,19 @@
         <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>78200</v>
       </c>
@@ -653,16 +677,19 @@
         <v>5</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>78600</v>
       </c>
@@ -670,16 +697,19 @@
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>78700</v>
       </c>
@@ -687,16 +717,19 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>79100</v>
       </c>
@@ -704,16 +737,19 @@
         <v>5</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>78800</v>
       </c>
@@ -721,16 +757,19 @@
         <v>5</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>73800</v>
       </c>
@@ -738,16 +777,19 @@
         <v>5</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>74100</v>
       </c>
@@ -755,16 +797,19 @@
         <v>17</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>78400</v>
       </c>
@@ -772,16 +817,19 @@
         <v>17</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>77700</v>
       </c>
@@ -789,16 +837,19 @@
         <v>17</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>76400</v>
       </c>
@@ -806,16 +857,19 @@
         <v>17</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>73500</v>
       </c>
@@ -823,16 +877,19 @@
         <v>17</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>76700</v>
       </c>
@@ -840,16 +897,19 @@
         <v>17</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>76500</v>
       </c>
@@ -857,16 +917,19 @@
         <v>17</v>
       </c>
       <c r="C17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>73600</v>
       </c>
@@ -874,16 +937,19 @@
         <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>77900</v>
       </c>
@@ -891,16 +957,19 @@
         <v>27</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>79400</v>
       </c>
@@ -908,16 +977,19 @@
         <v>27</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>78950</v>
       </c>
@@ -925,16 +997,19 @@
         <v>27</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>78900</v>
       </c>
@@ -942,16 +1017,19 @@
         <v>27</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>79600</v>
       </c>
@@ -959,16 +1037,19 @@
         <v>27</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>71300</v>
       </c>
@@ -976,16 +1057,19 @@
         <v>27</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>79700</v>
       </c>
@@ -993,16 +1077,19 @@
         <v>27</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>79500</v>
       </c>
@@ -1010,16 +1097,19 @@
         <v>27</v>
       </c>
       <c r="C26" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="F26" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>77500</v>
       </c>
@@ -1027,16 +1117,19 @@
         <v>27</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>79300</v>
       </c>
@@ -1044,16 +1137,19 @@
         <v>27</v>
       </c>
       <c r="C28" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>73700</v>
       </c>
@@ -1061,12 +1157,15 @@
         <v>27</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="E29" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>